<commit_message>
feat(validation): enforce mandatory Call Date on HR Called=Yes and add Not Interested tracking support
</commit_message>
<xml_diff>
--- a/candidates_tracker.xlsx
+++ b/candidates_tracker.xlsx
@@ -521,52 +521,52 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Actively Looking</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Resume_Aarav.pdf</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-30 18:00:00</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Resume_Aarav.pdf</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Naukri</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>sample_resume_aarav.pdf</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-08-24 08:57:48</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>sample_resume_aarav.pdf</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Android mobile verified at 08:58:52: Box items scroll and fit screen perfectly.</t>
+          <t>Playwright Screening: Candidate verified for next stage.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Follow up on technical screening</t>
+          <t>Technical interview scheduled with Lead</t>
         </is>
       </c>
     </row>
@@ -598,52 +598,52 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>Serving Notice</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Naukri.com</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Resume_Priya.pdf</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-08-30 18:15:00</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Resume_Priya.pdf</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>sample_resume_priya.pdf</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-08-24 08:57:48</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>sample_resume_priya.pdf</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Interested in Lead Full-Stack position</t>
+          <t>Notice period 30 days. Requested package details.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Interview scheduled with Tech Lead</t>
+          <t>Share company profile and JD</t>
         </is>
       </c>
     </row>
@@ -675,59 +675,49 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not Interested</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Indeed India</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>sample_resume_vikram.pdf</t>
+          <t>Resume_Vikram.pdf</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-08-24 08:57:48</t>
+          <t>2026-08-30 18:30:00</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>sample_resume_vikram.pdf</t>
+          <t>Resume_Vikram.pdf</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes - Not Interested</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>DevOps &amp; Cloud architecture specialist</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Verify notice period</t>
+          <t>Not interested in relocation to Bengaluru. Looking for remote only.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ananya Rao</t>
+          <t>Neha Verma</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -737,7 +727,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ananya.rao@example.com</t>
+          <t>neha.verma@example.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -747,32 +737,32 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3 Years</t>
+          <t>3.5 Years</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Actively Looking</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Naukri</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>sample_resume_ananya.pdf</t>
+          <t>Resume_Neha.pdf</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-24 08:57:48</t>
+          <t>2026-08-30 18:45:00</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>sample_resume_ananya.pdf</t>
+          <t>Resume_Neha.pdf</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -780,31 +770,16 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Frontend React &amp; UI/UX specialist</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Send technical take-home assignment</t>
+          <t>Candidate profile shortlisted for QA Automation.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Rohan Mehta</t>
+          <t>Rohan Kulkarni</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -814,67 +789,67 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>rohan.mehta@example.com</t>
+          <t>rohan.kulkarni@example.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Delhi NCR, India</t>
+          <t>Chennai, India</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>7 Years</t>
+          <t>8 Years</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Actively Looking</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Google / Web Search</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>sample_resume_rohan.pdf</t>
+          <t>Resume_Rohan.pdf</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-24 08:57:48</t>
+          <t>2026-08-30 19:00:00</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>sample_resume_rohan.pdf</t>
+          <t>Resume_Rohan.pdf</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Busy / Call Later</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>AI/ML Systems Architect</t>
+          <t>Candidate requested call back tomorrow after 4 PM.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Executive round in progress</t>
+          <t>Follow-up call at 4:30 PM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(escalation): add 4-tier escalation matrix (L1-L4), action categories, comments, Excel sync, and filter support
</commit_message>
<xml_diff>
--- a/candidates_tracker.xlsx
+++ b/candidates_tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,6 +492,21 @@
           <t>HR Follow-up Remarks</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Escalation Level / Person</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Escalation Action Category</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Escalation Remarks</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -556,7 +571,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Playwright Screening: Candidate verified for next stage.</t>
+          <t>Android mobile verified at 00:47:41: Box items scroll and fit screen perfectly.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -567,6 +582,21 @@
       <c r="O2" t="inlineStr">
         <is>
           <t>Technical interview scheduled with Lead</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>L2 - Raj</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Review / Suggest</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Escalated to L2 Raj: Review candidate Python experience and suggest compensation.</t>
         </is>
       </c>
     </row>

</xml_diff>